<commit_message>
Tuần 4: phân tích văn bản, word cloud, phát hiện Deal
</commit_message>
<xml_diff>
--- a/docs/Tracking_DAP391m.xlsx
+++ b/docs/Tracking_DAP391m.xlsx
@@ -988,7 +988,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Hoàn thiện notebook 00, 06, cập nhật README và tracking
</commit_message>
<xml_diff>
--- a/docs/Tracking_DAP391m.xlsx
+++ b/docs/Tracking_DAP391m.xlsx
@@ -1248,7 +1248,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Gắn nhãn cho các tin đăng bằng mô hình chính thức từ notebook 05; thống kê theo nhãn; case study trên tin thực tế; error analysis các tin lệch nhiều</t>
+          <t>Gắn nhãn cho các tin test bằng mô hình chính thức từ notebook 05; thống kê theo nhãn, khu vực, hãng; case study trên tin thực tế; dùng sai số theo khoảng giá của notebook 05 để đánh giá nhãn (không tính lại phân tích sai số)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Thống kê số tin theo từng nhãn; case study kiểm chứng được bằng tin thật; chỉ ra phân khúc mô hình hay sai</t>
+          <t>Thống kê số tin theo từng nhãn; case study kiểm chứng được bằng tin thật; dùng lại kết quả sai số của notebook 05</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Hoàn thiện form định giá, kiểm tra T21
</commit_message>
<xml_diff>
--- a/docs/Tracking_DAP391m.xlsx
+++ b/docs/Tracking_DAP391m.xlsx
@@ -587,7 +587,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>15.000 → 13.614 tin sau lọc IQR (loại 9,24%)</t>
+          <t>15.000 → 13.520 tin sau làm sạch (loại 9,87%), đối chiếu cars_cleaned.csv</t>
         </is>
       </c>
     </row>
@@ -911,17 +911,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>03 · Phân tích trực quan</t>
+          <t>06 · Dashboard trong notebook</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>hiển thị lọc theo hãng, dòng xe, tỉnh, khoảng năm</t>
+          <t>Dashboard nhập thông số định giá ngay trong notebook 06; hãng–dòng phụ thuộc, gợi ý theo hãng–dòng–năm có xác nhận</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Quách Thiện Nhân</t>
+          <t>Nguyễn Huy Sơn</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Tuần 4</t>
+          <t>Tuần 6</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -941,17 +941,17 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T15, T18</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>02_analytics_and_dashboard/dashboard.ipynb</t>
+          <t>03_nlp_and_deal/06_phat_hien_deal.ipynb</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Đổi bộ lọc thì biểu đồ cập nhật; kết luận chính vẫn có ở các biểu đồ tĩnh</t>
+          <t>Đã kiểm tra bằng test_dinh_gia.py và Jupyter trên máy hiện tại: hãng–dòng đúng, gợi ý có xác nhận, đầu vào sai bị chặn, định giá trả kết quả; chạy lại notebook để tương tác</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Chọn đặc trưng, mã hóa biến danh mục (One-Hot, xử lý 422 dòng xe), chia train/test 80/20 với random_state=42 trong Pipeline scikit-learn; huấn luyện Linear Regression (baseline), Decision Tree, Random Forest, XGBoost</t>
+          <t>Chọn 21 đặc trưng, mã hóa biến danh mục (422 dòng xe gốc, 372 sau làm sạch), chia train/test 80/20 với random_state=42; huấn luyện Linear Regression, Decision Tree, Random Forest, XGBoost trong Pipeline</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T06, T12</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Mỗi insight có số liệu minh chứng và ý nghĩa với người mua/người bán</t>
+          <t>Mục 8 notebook 03 có phép tính kiểm chứng và ý nghĩa với người mua/người bán; nhận xét bản đồ khớp tập sạch</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1518,12 +1518,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Toàn bộ repo</t>
+          <t>Toàn bộ repo + docs/T21_result.json</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Chạy lại không lỗi trên máy thành viên khác; số liệu giữa các notebook khớp nhau</t>
+          <t>Theo yêu cầu Sơn: nghiệm thu trên máy Sơn ngày 21/10/2026; chạy đủ 8 notebook trong bản sao tạm từ dữ liệu thô có sẵn, gồm làm sạch/NLP/huấn luyện; dữ liệu và dự đoán tái tạo khớp. Không xác nhận máy khác; không cào lại. Xem docs/T21_result.json</t>
         </is>
       </c>
     </row>
@@ -1535,12 +1535,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Bảo vệ</t>
+          <t>Hoàn thiện</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Chuẩn hóa repo (README, PEP8), thiết kế slide thuyết trình và phân chia lượt nói</t>
+          <t>Rà soát README, cấu trúc repo và sản phẩm bàn giao theo proposal</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1570,12 +1570,12 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Slide PPTX + GitHub repo</t>
+          <t>GitHub repo + notebooks</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Slide chuyên nghiệp, phân chia lượt nói cân đối</t>
+          <t>README khớp thực tế; sản phẩm bàn giao đủ theo proposal</t>
         </is>
       </c>
     </row>

</xml_diff>